<commit_message>
fix: corregir trazabilidad y metadatos de publicacion
</commit_message>
<xml_diff>
--- a/data/raw_equipo/ENVs.xlsx
+++ b/data/raw_equipo/ENVs.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonat\OneDrive\Documentos\MOOOONOGRAFIA\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{E15FBEA3-B339-422D-B3A3-4C11EE68A7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>